<commit_message>
chore(project): regenerate the artefacts from the current schema
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/spdx_linkml.xlsx
+++ b/project/excel/spdx_linkml.xlsx
@@ -483,47 +483,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -595,47 +595,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -701,47 +701,47 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -811,47 +811,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -928,47 +928,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1060,47 +1060,47 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1136,47 +1136,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1197,14 +1197,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>annotationType</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>contentType</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>annotationType</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
           <t>statement</t>
@@ -1227,53 +1227,53 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"other,review"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1333,47 +1333,47 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1409,47 +1409,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1525,47 +1525,47 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1668,47 +1668,47 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1744,47 +1744,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1881,29 +1881,29 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="M1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -1926,47 +1926,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2045,29 +2045,29 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="P1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2090,47 +2090,47 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2186,47 +2186,47 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2287,47 +2287,47 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2396,29 +2396,29 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="N1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2441,47 +2441,47 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2632,29 +2632,29 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="AE1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2677,47 +2677,47 @@
       </c>
       <c r="AI1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2939,29 +2939,29 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="AC1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2984,47 +2984,47 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3077,47 +3077,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3138,39 +3138,39 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>isDeprecatedLicenseId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>isFsfLibre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>isOsiApproved</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>licenseText</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>isDeprecatedLicenseId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>isFsfLibre</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>isOsiApproved</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>standardLicenseHeader</t>
@@ -3193,47 +3193,47 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3254,29 +3254,29 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>additionText</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>isDeprecatedAdditionId</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>additionText</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>isDeprecatedAdditionId</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
           <t>standardAdditionTemplate</t>
@@ -3294,47 +3294,47 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3370,47 +3370,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3461,47 +3461,47 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3537,47 +3537,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3608,39 +3608,39 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>isDeprecatedLicenseId</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>isFsfLibre</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>isOsiApproved</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>licenseText</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>isDeprecatedLicenseId</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>isFsfLibre</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>isOsiApproved</t>
-        </is>
-      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>standardLicenseHeader</t>
@@ -3663,47 +3663,47 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3734,29 +3734,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>additionText</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>isDeprecatedAdditionId</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>additionText</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>isDeprecatedAdditionId</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>standardAdditionTemplate</t>
@@ -3774,47 +3774,47 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3850,47 +3850,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3931,47 +3931,47 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4002,29 +4002,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4067,47 +4067,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4148,29 +4148,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4213,47 +4213,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4297,29 +4297,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4362,47 +4362,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4441,29 +4441,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4506,47 +4506,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4587,29 +4587,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4652,47 +4652,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4772,29 +4772,29 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4837,47 +4837,47 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4926,29 +4926,29 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4991,47 +4991,47 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5067,29 +5067,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -5132,47 +5132,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5223,29 +5223,29 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="K1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -5288,47 +5288,47 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5367,29 +5367,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -5432,47 +5432,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5513,29 +5513,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -5558,47 +5558,47 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5711,22 +5711,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>definingArtifact</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>externalSpdxId</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>locationHint</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>definingArtifact</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>externalSpdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>locationHint</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(project): regenerate the artefacts from the current schema (#21)
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/spdx_linkml.xlsx
+++ b/project/excel/spdx_linkml.xlsx
@@ -483,47 +483,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -595,47 +595,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -701,47 +701,47 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -811,47 +811,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -928,47 +928,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1060,47 +1060,47 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1136,47 +1136,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1197,14 +1197,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>annotationType</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>contentType</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>annotationType</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
           <t>statement</t>
@@ -1227,53 +1227,53 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"other,review"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1333,47 +1333,47 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1409,47 +1409,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1525,47 +1525,47 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1668,47 +1668,47 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1744,47 +1744,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -1881,29 +1881,29 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="M1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -1926,47 +1926,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2045,29 +2045,29 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="P1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2090,47 +2090,47 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2186,47 +2186,47 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2287,47 +2287,47 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2396,29 +2396,29 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="N1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2441,47 +2441,47 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2632,29 +2632,29 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="AE1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2677,47 +2677,47 @@
       </c>
       <c r="AI1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -2939,29 +2939,29 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="AC1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -2984,47 +2984,47 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3077,47 +3077,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3138,39 +3138,39 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>isDeprecatedLicenseId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>isFsfLibre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>isOsiApproved</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>licenseText</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>isDeprecatedLicenseId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>isFsfLibre</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>isOsiApproved</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>standardLicenseHeader</t>
@@ -3193,47 +3193,47 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3254,29 +3254,29 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>additionText</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>isDeprecatedAdditionId</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>additionText</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>isDeprecatedAdditionId</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
           <t>standardAdditionTemplate</t>
@@ -3294,47 +3294,47 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3370,47 +3370,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3461,47 +3461,47 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3537,47 +3537,47 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3608,39 +3608,39 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>isDeprecatedLicenseId</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>isFsfLibre</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>isOsiApproved</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>licenseText</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>isDeprecatedLicenseId</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>isFsfLibre</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>isOsiApproved</t>
-        </is>
-      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>standardLicenseHeader</t>
@@ -3663,47 +3663,47 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3734,29 +3734,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>additionText</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>isDeprecatedAdditionId</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>licenseXml</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>obsoletedBy</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>seeAlso</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>additionText</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>isDeprecatedAdditionId</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>standardAdditionTemplate</t>
@@ -3774,47 +3774,47 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3850,47 +3850,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -3931,47 +3931,47 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4002,29 +4002,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4067,47 +4067,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4148,29 +4148,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4213,47 +4213,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4297,29 +4297,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4362,47 +4362,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4441,29 +4441,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4506,47 +4506,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4587,29 +4587,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4652,47 +4652,47 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4772,29 +4772,29 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4837,47 +4837,47 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -4926,29 +4926,29 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -4991,47 +4991,47 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5067,29 +5067,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -5132,47 +5132,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5223,29 +5223,29 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="K1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -5288,47 +5288,47 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5367,29 +5367,29 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>assessedElement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>modifiedTime</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>publishedTime</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>withdrawnTime</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assessedElement</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
           <t>completeness</t>
@@ -5432,47 +5432,47 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5513,29 +5513,29 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>builtTime</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>originatedBy</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>releaseTime</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>standardName</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>suppliedBy</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>builtTime</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>originatedBy</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>releaseTime</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>standardName</t>
-        </is>
-      </c>
       <c r="I1" t="inlineStr">
         <is>
           <t>supportLevel</t>
@@ -5558,47 +5558,47 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>creationInfo</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>externalIdentifier</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>externalRef</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>spdxId</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>creationInfo</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>extension</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>externalIdentifier</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>externalRef</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>summary</t>
         </is>
       </c>
     </row>
@@ -5711,22 +5711,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>definingArtifact</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>externalSpdxId</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>locationHint</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>verifiedUsing</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>definingArtifact</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>externalSpdxId</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>locationHint</t>
         </is>
       </c>
     </row>

</xml_diff>